<commit_message>
Created the DataProvider Util for the Excel data that is used in create job api test
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -8,10 +8,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateJobTestData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr/>
 </workbook>
@@ -30,6 +31,144 @@
   </si>
   <si>
     <t>iamsup</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>jay</t>
+  </si>
+  <si>
+    <t>Bernhard</t>
+  </si>
+  <si>
+    <t>919-337-0053</t>
+  </si>
+  <si>
+    <t>Roberto35@yahoo.com</t>
+  </si>
+  <si>
+    <t>c 304</t>
+  </si>
+  <si>
+    <t>Jupiter</t>
+  </si>
+  <si>
+    <t>MG road</t>
+  </si>
+  <si>
+    <t>Bangur Nagar</t>
+  </si>
+  <si>
+    <t>Goregaon West</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>56372684145597</t>
+  </si>
+  <si>
+    <t>Battery Issue</t>
+  </si>
+  <si>
+    <t>Ajay</t>
+  </si>
+  <si>
+    <t>46372684145596</t>
+  </si>
+  <si>
+    <t>Dnyaneshwar</t>
+  </si>
+  <si>
+    <t>36372684145596</t>
+  </si>
+  <si>
+    <t>Deepak</t>
+  </si>
+  <si>
+    <t>26372684145596</t>
   </si>
 </sst>
 </file>
@@ -73,9 +212,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -376,4 +518,445 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.42578" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.71094" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.28516" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85547" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.57031" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.85547" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.71094" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.28516" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.14063" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.42578" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.42578" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.42578" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.28516" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="25.85547" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.57031" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.57031" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.14063" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.14063" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="28.71094" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.85547" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.14063" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.71094" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="1">
+        <v>411039</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="3">
+        <v>45754</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="W2" s="3">
+        <v>45754</v>
+      </c>
+      <c r="X2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="1">
+        <v>411039</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" s="3">
+        <v>45754</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" s="3">
+        <v>45754</v>
+      </c>
+      <c r="X3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" s="1">
+        <v>411039</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="3">
+        <v>45754</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="W4" s="3">
+        <v>45754</v>
+      </c>
+      <c r="X4" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>0</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="1">
+        <v>411039</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" s="3">
+        <v>45754</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="W5" s="3">
+        <v>45754</v>
+      </c>
+      <c r="X5" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB5" s="1"/>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>